<commit_message>
ci: update with stable _record_id for split records
- Updated docs/index.html with 389 records (DHD_1, DHD_2, GEX_1, GEX_2)
- Updated index.html with same embedded data
- Updated web/vps_automation_vhck.html with same embedded data
- Updated data/vsd_records.json with _record_id field
- Updated data/vsd_records.xlsx with new records
- All split records have unique, stable IDs across runs

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/vsd_records.xlsx
+++ b/data/vsd_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD390"/>
+  <dimension ref="A1:AE390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -444,8 +444,9 @@
     <col width="37" customWidth="1" min="26" max="26"/>
     <col width="10" customWidth="1" min="27" max="27"/>
     <col width="50" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="21" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,10 +592,15 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>_record_id</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>mã_chứng_khoán</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>confirmation_status</t>
         </is>
@@ -694,8 +700,13 @@
 22/04/2026</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>E1VFVN30</t>
+        </is>
+      </c>
       <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -838,8 +849,13 @@
 CTCP Vật Tư Bưu Điện và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng chứng khoán đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>PMJ</t>
+        </is>
+      </c>
       <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -988,8 +1004,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>NLG12404</t>
+        </is>
+      </c>
       <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1162,8 +1183,13 @@
 Công ty cổ phần X20 và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>X20</t>
+        </is>
+      </c>
       <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1315,8 +1341,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>ASG12501</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1459,8 +1490,13 @@
 Công ty Cổ phần Chế tạo Biến thế và Vật liệu điện Hà Nội và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>BTH</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1603,8 +1639,13 @@
 Công ty cổ phần BOT Cầu Thái Hà và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1741,8 +1782,13 @@
 Công ty cổ phần Phân lân Ninh Bình và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>NFC</t>
+        </is>
+      </c>
       <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1885,8 +1931,13 @@
 Công ty cổ phần Xây dựng 1369 và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>C69</t>
+        </is>
+      </c>
       <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2029,8 +2080,13 @@
 Công ty Cổ phần Sữa Hà Nội và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>HNM</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2173,8 +2229,13 @@
 Công ty cổ phần Đầu tư Bitco Bình Định và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2315,8 +2376,13 @@
 Công ty cổ phần Bia Sài Gòn - Miền Trung, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
+      </c>
       <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2430,8 +2496,13 @@
 VSDC thông báo để các Thành viên lưu ký biết và thực hiện./.</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>VHM12404</t>
+        </is>
+      </c>
       <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2494,8 +2565,13 @@
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>XD312301</t>
+        </is>
+      </c>
       <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2642,8 +2718,13 @@
 CTCP Vận tải Dầu khí Thái Bình Dương, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>PVP</t>
+        </is>
+      </c>
       <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2706,8 +2787,13 @@
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>PVP</t>
+        </is>
+      </c>
       <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2850,8 +2936,13 @@
 Công ty Cổ phần Kỹ nghệ Khoáng sản Quảng Nam, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>MIC</t>
+        </is>
+      </c>
       <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2994,8 +3085,13 @@
 CTCP Bất động sản cho thuê Minh Bảo Tín và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>MBT</t>
+        </is>
+      </c>
       <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3140,8 +3236,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>ABB12509</t>
+        </is>
+      </c>
       <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3286,8 +3387,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>ABB12508</t>
+        </is>
+      </c>
       <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3383,8 +3489,13 @@
 22/04/2026</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>FUEVFVND</t>
+        </is>
+      </c>
       <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3480,8 +3591,13 @@
 22/04/2026</t>
         </is>
       </c>
-      <c r="AC23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>FUEVN100</t>
+        </is>
+      </c>
       <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3576,8 +3692,13 @@
 22/04/2026</t>
         </is>
       </c>
-      <c r="AC24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>FUESSV30</t>
+        </is>
+      </c>
       <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3640,8 +3761,13 @@
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>SHS12502</t>
+        </is>
+      </c>
       <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3756,8 +3882,13 @@
 CNVSDC thông báo để các Thành viên lưu ký biết và thực hiện./.</t>
         </is>
       </c>
-      <c r="AC26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>SPJ12101</t>
+        </is>
+      </c>
       <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3906,8 +4037,13 @@
 Công ty cổ phần Dược Vật tư Y tế Hải Dương và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>DHD_1</t>
+        </is>
+      </c>
       <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4057,8 +4193,13 @@
 Công ty cổ phần Dược Vật tư Y tế Hải Dương và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>DHD_2</t>
+        </is>
+      </c>
       <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4201,8 +4342,13 @@
 Công ty cổ phần Vàng Lào Cai và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>GLC</t>
+        </is>
+      </c>
       <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4339,8 +4485,13 @@
 Công ty cổ phần Tập đoàn Macstar và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
       <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4483,8 +4634,13 @@
 Công ty cổ phần Freco Việt Nam và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
       <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4633,8 +4789,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>BID12409</t>
+        </is>
+      </c>
       <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4783,8 +4944,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>BID12407</t>
+        </is>
+      </c>
       <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4919,8 +5085,13 @@
 Công ty cổ phần Tập đoàn CMH Việt Nam và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
       <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5082,8 +5253,13 @@
 Công ty cổ phần Tập đoàn BGI và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>VC7</t>
+        </is>
+      </c>
       <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5226,8 +5402,13 @@
 Công ty cổ phần CNC Capital Việt Nam và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>KSQ</t>
+        </is>
+      </c>
       <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5370,8 +5551,13 @@
 Công Ty Cổ Phần Vinafco và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>VFC</t>
+        </is>
+      </c>
       <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5516,8 +5702,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>PC112202</t>
+        </is>
+      </c>
       <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5660,8 +5851,13 @@
 CTCP Cấp nước Cà Mau và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>CMW</t>
+        </is>
+      </c>
       <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5804,8 +6000,13 @@
 CTCP Nông súc sản Đồng Nai và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>NSS</t>
+        </is>
+      </c>
       <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5948,8 +6149,13 @@
 CTCP Khoáng sản và Xây dựng Bình Dương và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>KSB</t>
+        </is>
+      </c>
       <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6081,8 +6287,13 @@
 Công ty cổ phần ANI, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>ANI</t>
+        </is>
+      </c>
       <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6225,8 +6436,13 @@
 CTCP Cảng An Giang và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng chứng khoán đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>CAG</t>
+        </is>
+      </c>
       <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6384,8 +6600,13 @@
 Công ty cổ phần Camimex Group, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>CMX</t>
+        </is>
+      </c>
       <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6536,8 +6757,13 @@
 Công ty cổ phần Tập đoàn GELEX, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>GEX_1</t>
+        </is>
+      </c>
       <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6688,8 +6914,13 @@
 Công ty cổ phần Tập đoàn GELEX, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>GEX_2</t>
+        </is>
+      </c>
       <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6829,8 +7060,13 @@
 Công ty cổ phần Sách và Thiết bị Trường học Quảng Ninh và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>QST</t>
+        </is>
+      </c>
       <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6974,8 +7210,13 @@
 Công ty cổ phần BV Land và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>BVL</t>
+        </is>
+      </c>
       <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7118,8 +7359,13 @@
 Công ty cổ phần Bảo hiểm Ngân hàng Nông nghiệp và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>ABI</t>
+        </is>
+      </c>
       <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7254,8 +7500,13 @@
 Công ty cổ phần SIVICO và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>SIV</t>
+        </is>
+      </c>
       <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7412,8 +7663,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>BID12406</t>
+        </is>
+      </c>
       <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7565,8 +7821,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>VIF12501</t>
+        </is>
+      </c>
       <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7723,8 +7984,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>BID12408</t>
+        </is>
+      </c>
       <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7867,8 +8133,13 @@
 Công ty cổ phần Vận tải hóa dầu VP và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>VPA</t>
+        </is>
+      </c>
       <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8006,8 +8277,13 @@
 Công ty Cổ phần Đầu tư và Thương mại TNG và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>TNG</t>
+        </is>
+      </c>
       <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8150,8 +8426,13 @@
 Công ty cổ phần Thực phẩm Hữu Nghị và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>HNF</t>
+        </is>
+      </c>
       <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8287,8 +8568,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>LPB126020</t>
+        </is>
+      </c>
       <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8424,8 +8710,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>LPB126019</t>
+        </is>
+      </c>
       <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8561,8 +8852,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>LPB126018</t>
+        </is>
+      </c>
       <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8699,8 +8995,13 @@
 Công ty cổ phần Điện lực Gelex và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>GEE</t>
+        </is>
+      </c>
       <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8808,8 +9109,13 @@
 Công ty cổ phần Phát triển hạ tầng Vĩnh Phúc và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng chứng khoán đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>IDV</t>
+        </is>
+      </c>
       <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8952,8 +9258,13 @@
 Công ty Cổ Phần Tập đoàn Green+, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>GPC</t>
+        </is>
+      </c>
       <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9095,8 +9406,13 @@
 CTCP Gạch Men Thanh Thanh, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>TTC</t>
+        </is>
+      </c>
       <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9245,8 +9561,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>VNG12401</t>
+        </is>
+      </c>
       <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9377,8 +9698,13 @@
 Công ty cổ phần Thực phẩm Sao Ta, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>FMC</t>
+        </is>
+      </c>
       <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9516,8 +9842,13 @@
 CTCP Tân Cảng - Phú Hữu và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>PNP</t>
+        </is>
+      </c>
       <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9660,8 +9991,13 @@
 CTCP Dịch vụ Du lịch Bến Thành, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>BTV</t>
+        </is>
+      </c>
       <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9804,8 +10140,13 @@
 Công ty cổ phần Tập đoàn VNG, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>VNZ</t>
+        </is>
+      </c>
       <c r="AD68" t="inlineStr"/>
+      <c r="AE68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9954,8 +10295,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>BID12507</t>
+        </is>
+      </c>
       <c r="AD69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10111,8 +10457,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC.</t>
         </is>
       </c>
-      <c r="AC70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>OCB12504</t>
+        </is>
+      </c>
       <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10261,8 +10612,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>BID12508</t>
+        </is>
+      </c>
       <c r="AD71" t="inlineStr"/>
+      <c r="AE71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10418,8 +10774,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC.</t>
         </is>
       </c>
-      <c r="AC72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>OCB12503</t>
+        </is>
+      </c>
       <c r="AD72" t="inlineStr"/>
+      <c r="AE72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10571,8 +10932,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>BID12506</t>
+        </is>
+      </c>
       <c r="AD73" t="inlineStr"/>
+      <c r="AE73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10724,8 +11090,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>BID12116</t>
+        </is>
+      </c>
       <c r="AD74" t="inlineStr"/>
+      <c r="AE74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10868,8 +11239,13 @@
 Tập đoàn Công nghiệp Cao su Việt Nam - CTCP và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>GVR</t>
+        </is>
+      </c>
       <c r="AD75" t="inlineStr"/>
+      <c r="AE75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -11012,8 +11388,13 @@
 Công ty cổ phần Đầu tư Phát triển Công nghiệp – Thương mại Củ Chi, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>CCI</t>
+        </is>
+      </c>
       <c r="AD76" t="inlineStr"/>
+      <c r="AE76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -11175,8 +11556,13 @@
 CTCP Camimex và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
       <c r="AD77" t="inlineStr"/>
+      <c r="AE77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -11311,8 +11697,13 @@
 Công ty cổ phần Thủy Đặc Sản và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>SPV</t>
+        </is>
+      </c>
       <c r="AD78" t="inlineStr"/>
+      <c r="AE78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -11375,8 +11766,13 @@
       <c r="Z79" t="inlineStr"/>
       <c r="AA79" t="inlineStr"/>
       <c r="AB79" t="inlineStr"/>
-      <c r="AC79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>BPB12101</t>
+        </is>
+      </c>
       <c r="AD79" t="inlineStr"/>
+      <c r="AE79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -11525,8 +11921,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>BID12405</t>
+        </is>
+      </c>
       <c r="AD80" t="inlineStr"/>
+      <c r="AE80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -11671,8 +12072,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>LHT12401</t>
+        </is>
+      </c>
       <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -11821,8 +12227,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC82" t="inlineStr"/>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>TCB12509</t>
+        </is>
+      </c>
       <c r="AD82" t="inlineStr"/>
+      <c r="AE82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -11971,8 +12382,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC83" t="inlineStr"/>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>TCB12508</t>
+        </is>
+      </c>
       <c r="AD83" t="inlineStr"/>
+      <c r="AE83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -12111,8 +12527,13 @@
 Ngân hàng Thương mại cổ phần Quốc tế Việt Nam và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC84" t="inlineStr"/>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>VIB</t>
+        </is>
+      </c>
       <c r="AD84" t="inlineStr"/>
+      <c r="AE84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -12208,8 +12629,13 @@
 20/04/2026</t>
         </is>
       </c>
-      <c r="AC85" t="inlineStr"/>
+      <c r="AC85" t="inlineStr">
+        <is>
+          <t>E1VFVN30</t>
+        </is>
+      </c>
       <c r="AD85" t="inlineStr"/>
+      <c r="AE85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -12353,8 +12779,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC86" t="inlineStr"/>
+      <c r="AC86" t="inlineStr">
+        <is>
+          <t>NTJ12601</t>
+        </is>
+      </c>
       <c r="AD86" t="inlineStr"/>
+      <c r="AE86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12499,8 +12930,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC87" t="inlineStr"/>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>VHM12601</t>
+        </is>
+      </c>
       <c r="AD87" t="inlineStr"/>
+      <c r="AE87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -12636,8 +13072,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC88" t="inlineStr"/>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>HDB126017</t>
+        </is>
+      </c>
       <c r="AD88" t="inlineStr"/>
+      <c r="AE88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12773,8 +13214,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC89" t="inlineStr"/>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>HDB126016</t>
+        </is>
+      </c>
       <c r="AD89" t="inlineStr"/>
+      <c r="AE89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -12869,8 +13315,13 @@
 20/04/2026</t>
         </is>
       </c>
-      <c r="AC90" t="inlineStr"/>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>FUEVFVND</t>
+        </is>
+      </c>
       <c r="AD90" t="inlineStr"/>
+      <c r="AE90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -13013,8 +13464,13 @@
 Công ty cổ phần Xi măng Phú Thọ và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC91" t="inlineStr"/>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>PTE</t>
+        </is>
+      </c>
       <c r="AD91" t="inlineStr"/>
+      <c r="AE91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -13157,8 +13613,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC92" t="inlineStr"/>
+      <c r="AC92" t="inlineStr">
+        <is>
+          <t>VJC12332</t>
+        </is>
+      </c>
       <c r="AD92" t="inlineStr"/>
+      <c r="AE92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -13297,8 +13758,13 @@
 Công ty cổ phần Vimarko và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC93" t="inlineStr"/>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>VMK</t>
+        </is>
+      </c>
       <c r="AD93" t="inlineStr"/>
+      <c r="AE93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -13441,8 +13907,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC94" t="inlineStr"/>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>VJC12331</t>
+        </is>
+      </c>
       <c r="AD94" t="inlineStr"/>
+      <c r="AE94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -13591,8 +14062,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC.</t>
         </is>
       </c>
-      <c r="AC95" t="inlineStr"/>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>BAF12501</t>
+        </is>
+      </c>
       <c r="AD95" t="inlineStr"/>
+      <c r="AE95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -13760,8 +14236,13 @@
 Công ty Cổ phần Bến xe Miền Tây, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC96" t="inlineStr"/>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>WCS</t>
+        </is>
+      </c>
       <c r="AD96" t="inlineStr"/>
+      <c r="AE96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13824,8 +14305,13 @@
       <c r="Z97" t="inlineStr"/>
       <c r="AA97" t="inlineStr"/>
       <c r="AB97" t="inlineStr"/>
-      <c r="AC97" t="inlineStr"/>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>TV6</t>
+        </is>
+      </c>
       <c r="AD97" t="inlineStr"/>
+      <c r="AE97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13962,8 +14448,13 @@
 Công ty cổ phần Dịch vụ Du lịch Phú Thọ, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC98" t="inlineStr"/>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
       <c r="AD98" t="inlineStr"/>
+      <c r="AE98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -14026,8 +14517,13 @@
       <c r="Z99" t="inlineStr"/>
       <c r="AA99" t="inlineStr"/>
       <c r="AB99" t="inlineStr"/>
-      <c r="AC99" t="inlineStr"/>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
       <c r="AD99" t="inlineStr"/>
+      <c r="AE99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -14180,8 +14676,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC100" t="inlineStr"/>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>VPB12505</t>
+        </is>
+      </c>
       <c r="AD100" t="inlineStr"/>
+      <c r="AE100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -14329,8 +14830,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC101" t="inlineStr"/>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>MBB12414</t>
+        </is>
+      </c>
       <c r="AD101" t="inlineStr"/>
+      <c r="AE101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -14475,8 +14981,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC102" t="inlineStr"/>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>TCB12403</t>
+        </is>
+      </c>
       <c r="AD102" t="inlineStr"/>
+      <c r="AE102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -14611,8 +15122,13 @@
 Công ty Cổ phần may xuất khẩu Phan Thiết, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC103" t="inlineStr"/>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>PTG</t>
+        </is>
+      </c>
       <c r="AD103" t="inlineStr"/>
+      <c r="AE103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -14795,8 +15311,13 @@
 CTCP Chiếu sáng công cộng TP. Hồ Chí Minh và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC104" t="inlineStr"/>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>CHS</t>
+        </is>
+      </c>
       <c r="AD104" t="inlineStr"/>
+      <c r="AE104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -14859,8 +15380,13 @@
       <c r="Z105" t="inlineStr"/>
       <c r="AA105" t="inlineStr"/>
       <c r="AB105" t="inlineStr"/>
-      <c r="AC105" t="inlineStr"/>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>PDV</t>
+        </is>
+      </c>
       <c r="AD105" t="inlineStr"/>
+      <c r="AE105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -14996,8 +15522,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC106" t="inlineStr"/>
+      <c r="AC106" t="inlineStr">
+        <is>
+          <t>MC3</t>
+        </is>
+      </c>
       <c r="AD106" t="inlineStr"/>
+      <c r="AE106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -15101,8 +15632,13 @@
 Công ty cổ phần Chứng khoán DNSE và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng cổ phiếu đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC107" t="inlineStr"/>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>DSE</t>
+        </is>
+      </c>
       <c r="AD107" t="inlineStr"/>
+      <c r="AE107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -15246,8 +15782,13 @@
 Công ty cổ phần Tư vấn thiết kế và Phát triển đô thị và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC108" t="inlineStr"/>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>CDO</t>
+        </is>
+      </c>
       <c r="AD108" t="inlineStr"/>
+      <c r="AE108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -15310,8 +15851,13 @@
       <c r="Z109" t="inlineStr"/>
       <c r="AA109" t="inlineStr"/>
       <c r="AB109" t="inlineStr"/>
-      <c r="AC109" t="inlineStr"/>
+      <c r="AC109" t="inlineStr">
+        <is>
+          <t>TMI12401</t>
+        </is>
+      </c>
       <c r="AD109" t="inlineStr"/>
+      <c r="AE109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -15407,8 +15953,13 @@
 17/04/2026</t>
         </is>
       </c>
-      <c r="AC110" t="inlineStr"/>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>FUEKIV30</t>
+        </is>
+      </c>
       <c r="AD110" t="inlineStr"/>
+      <c r="AE110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -15504,8 +16055,13 @@
 17/04/2026</t>
         </is>
       </c>
-      <c r="AC111" t="inlineStr"/>
+      <c r="AC111" t="inlineStr">
+        <is>
+          <t>E1VFVN30</t>
+        </is>
+      </c>
       <c r="AD111" t="inlineStr"/>
+      <c r="AE111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -15648,8 +16204,13 @@
 Tổng công ty May 10 - Công ty cổ phần và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC112" t="inlineStr"/>
+      <c r="AC112" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
       <c r="AD112" t="inlineStr"/>
+      <c r="AE112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -15712,8 +16273,13 @@
       <c r="Z113" t="inlineStr"/>
       <c r="AA113" t="inlineStr"/>
       <c r="AB113" t="inlineStr"/>
-      <c r="AC113" t="inlineStr"/>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
       <c r="AD113" t="inlineStr"/>
+      <c r="AE113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -15847,8 +16413,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC114" t="inlineStr"/>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>VKS12101</t>
+        </is>
+      </c>
       <c r="AD114" t="inlineStr"/>
+      <c r="AE114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -16000,8 +16571,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC115" t="inlineStr"/>
+      <c r="AC115" t="inlineStr">
+        <is>
+          <t>TPB12530</t>
+        </is>
+      </c>
       <c r="AD115" t="inlineStr"/>
+      <c r="AE115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -16153,8 +16729,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC116" t="inlineStr"/>
+      <c r="AC116" t="inlineStr">
+        <is>
+          <t>TPB12505</t>
+        </is>
+      </c>
       <c r="AD116" t="inlineStr"/>
+      <c r="AE116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -16288,8 +16869,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC117" t="inlineStr"/>
+      <c r="AC117" t="inlineStr">
+        <is>
+          <t>MIV12101</t>
+        </is>
+      </c>
       <c r="AD117" t="inlineStr"/>
+      <c r="AE117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -16439,8 +17025,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC118" t="inlineStr"/>
+      <c r="AC118" t="inlineStr">
+        <is>
+          <t>TPB12505</t>
+        </is>
+      </c>
       <c r="AD118" t="inlineStr"/>
+      <c r="AE118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -16575,8 +17166,13 @@
 Công ty cổ phần Đầu tư và Phát triển Giáo dục Hà Nội và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC119" t="inlineStr"/>
+      <c r="AC119" t="inlineStr">
+        <is>
+          <t>EID</t>
+        </is>
+      </c>
       <c r="AD119" t="inlineStr"/>
+      <c r="AE119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -16711,8 +17307,13 @@
 Công ty cổ phần Tập đoàn Đầu tư Din Capital và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC120" t="inlineStr"/>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>PDB</t>
+        </is>
+      </c>
       <c r="AD120" t="inlineStr"/>
+      <c r="AE120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -16855,8 +17456,13 @@
 Công ty cổ phần Cảng Đoạn Xá và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC121" t="inlineStr"/>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>DXP</t>
+        </is>
+      </c>
       <c r="AD121" t="inlineStr"/>
+      <c r="AE121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -16999,8 +17605,13 @@
 Công ty cổ phần Sản xuất - Xuất nhập khẩu Thanh Hà và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC122" t="inlineStr"/>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>HFX</t>
+        </is>
+      </c>
       <c r="AD122" t="inlineStr"/>
+      <c r="AE122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -17143,8 +17754,13 @@
 Công ty Cổ phần Sông Đà 6 và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC123" t="inlineStr"/>
+      <c r="AC123" t="inlineStr">
+        <is>
+          <t>SD6</t>
+        </is>
+      </c>
       <c r="AD123" t="inlineStr"/>
+      <c r="AE123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -17293,8 +17909,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC124" t="inlineStr"/>
+      <c r="AC124" t="inlineStr">
+        <is>
+          <t>HCH12401</t>
+        </is>
+      </c>
       <c r="AD124" t="inlineStr"/>
+      <c r="AE124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -17443,8 +18064,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC125" t="inlineStr"/>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>HCH12402</t>
+        </is>
+      </c>
       <c r="AD125" t="inlineStr"/>
+      <c r="AE125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -17540,8 +18166,13 @@
 17/04/2026</t>
         </is>
       </c>
-      <c r="AC126" t="inlineStr"/>
+      <c r="AC126" t="inlineStr">
+        <is>
+          <t>FUEDCMID</t>
+        </is>
+      </c>
       <c r="AD126" t="inlineStr"/>
+      <c r="AE126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -17637,8 +18268,13 @@
 17/04/2026</t>
         </is>
       </c>
-      <c r="AC127" t="inlineStr"/>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>FUEVN100</t>
+        </is>
+      </c>
       <c r="AD127" t="inlineStr"/>
+      <c r="AE127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -17775,8 +18411,13 @@
 Công ty cổ phần Quốc Cường Gia Lai, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ. Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC128" t="inlineStr"/>
+      <c r="AC128" t="inlineStr">
+        <is>
+          <t>QCG</t>
+        </is>
+      </c>
       <c r="AD128" t="inlineStr"/>
+      <c r="AE128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -17919,8 +18560,13 @@
 CTCP Công nghệ ITD và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC129" t="inlineStr"/>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>ITD</t>
+        </is>
+      </c>
       <c r="AD129" t="inlineStr"/>
+      <c r="AE129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -18064,8 +18710,13 @@
 Công ty cổ phần Đầu tư và Thương mại TNG, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC130" t="inlineStr"/>
+      <c r="AC130" t="inlineStr">
+        <is>
+          <t>TNG122017</t>
+        </is>
+      </c>
       <c r="AD130" t="inlineStr"/>
+      <c r="AE130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -18208,8 +18859,13 @@
 Công ty cổ phần Đầu tư và Thương mại TNG, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC131" t="inlineStr"/>
+      <c r="AC131" t="inlineStr">
+        <is>
+          <t>TNG124027</t>
+        </is>
+      </c>
       <c r="AD131" t="inlineStr"/>
+      <c r="AE131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -18352,8 +19008,13 @@
 Công ty cổ phần Vinhomes, tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào quá trình xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC132" t="inlineStr"/>
+      <c r="AC132" t="inlineStr">
+        <is>
+          <t>VHM121025</t>
+        </is>
+      </c>
       <c r="AD132" t="inlineStr"/>
+      <c r="AE132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -18498,8 +19159,13 @@
 0</t>
         </is>
       </c>
-      <c r="AC133" t="inlineStr"/>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>NAB12601</t>
+        </is>
+      </c>
       <c r="AD133" t="inlineStr"/>
+      <c r="AE133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -18670,8 +19336,13 @@
 Tổng Công ty Máy và Thiết bị Công nghiệp - CTCP và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC134" t="inlineStr"/>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>MIE</t>
+        </is>
+      </c>
       <c r="AD134" t="inlineStr"/>
+      <c r="AE134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -18806,8 +19477,13 @@
 Công ty cổ phần Thiết bị xăng dầu Petrolimex và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC135" t="inlineStr"/>
+      <c r="AC135" t="inlineStr">
+        <is>
+          <t>PEQ</t>
+        </is>
+      </c>
       <c r="AD135" t="inlineStr"/>
+      <c r="AE135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -18964,8 +19640,13 @@
 Công ty cổ phần Tập đoàn Sara và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC136" t="inlineStr"/>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>SRB</t>
+        </is>
+      </c>
       <c r="AD136" t="inlineStr"/>
+      <c r="AE136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -19121,8 +19802,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC137" t="inlineStr"/>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>BAB12501</t>
+        </is>
+      </c>
       <c r="AD137" t="inlineStr"/>
+      <c r="AE137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -19278,8 +19964,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC138" t="inlineStr"/>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>BAB12502</t>
+        </is>
+      </c>
       <c r="AD138" t="inlineStr"/>
+      <c r="AE138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -19432,8 +20123,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC139" t="inlineStr"/>
+      <c r="AC139" t="inlineStr">
+        <is>
+          <t>VPB12503</t>
+        </is>
+      </c>
       <c r="AD139" t="inlineStr"/>
+      <c r="AE139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -19585,8 +20281,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC140" t="inlineStr"/>
+      <c r="AC140" t="inlineStr">
+        <is>
+          <t>VPB12504</t>
+        </is>
+      </c>
       <c r="AD140" t="inlineStr"/>
+      <c r="AE140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -19738,8 +20439,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC141" t="inlineStr"/>
+      <c r="AC141" t="inlineStr">
+        <is>
+          <t>TPB12506</t>
+        </is>
+      </c>
       <c r="AD141" t="inlineStr"/>
+      <c r="AE141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -19882,8 +20588,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC142" t="inlineStr"/>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>SHD12404</t>
+        </is>
+      </c>
       <c r="AD142" t="inlineStr"/>
+      <c r="AE142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -20029,8 +20740,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC143" t="inlineStr"/>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>MBS12404</t>
+        </is>
+      </c>
       <c r="AD143" t="inlineStr"/>
+      <c r="AE143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -20177,8 +20893,13 @@
 CTCP Thủy Điện Cần Đơn và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC144" t="inlineStr"/>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>SJD</t>
+        </is>
+      </c>
       <c r="AD144" t="inlineStr"/>
+      <c r="AE144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -20324,8 +21045,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC145" t="inlineStr"/>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>MBS12301</t>
+        </is>
+      </c>
       <c r="AD145" t="inlineStr"/>
+      <c r="AE145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -20433,8 +21159,13 @@
 Công ty cổ phần Chứng khoán DSC và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng chứng khoán đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC146" t="inlineStr"/>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>DSC</t>
+        </is>
+      </c>
       <c r="AD146" t="inlineStr"/>
+      <c r="AE146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -20546,8 +21277,13 @@
 Công ty cổ phần Vận tải và Xếp dỡ Hải An và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin số lượng cổ phiếu đăng ký phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC147" t="inlineStr"/>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>HAH</t>
+        </is>
+      </c>
       <c r="AD147" t="inlineStr"/>
+      <c r="AE147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -20610,8 +21346,13 @@
       <c r="Z148" t="inlineStr"/>
       <c r="AA148" t="inlineStr"/>
       <c r="AB148" t="inlineStr"/>
-      <c r="AC148" t="inlineStr"/>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>BPG12101</t>
+        </is>
+      </c>
       <c r="AD148" t="inlineStr"/>
+      <c r="AE148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -20754,8 +21495,13 @@
 Công ty cổ phần Tập đoàn Tiên Sơn Thanh Hóa và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC149" t="inlineStr"/>
+      <c r="AC149" t="inlineStr">
+        <is>
+          <t>AAT</t>
+        </is>
+      </c>
       <c r="AD149" t="inlineStr"/>
+      <c r="AE149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -20922,8 +21668,13 @@
 Công ty cổ phần Đầu tư và Thương mại Dầu khí Nghệ An và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="AC150" t="inlineStr"/>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>PXA</t>
+        </is>
+      </c>
       <c r="AD150" t="inlineStr"/>
+      <c r="AE150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -21070,8 +21821,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC151" t="inlineStr"/>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>NPM12303</t>
+        </is>
+      </c>
       <c r="AD151" t="inlineStr"/>
+      <c r="AE151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -21218,8 +21974,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC152" t="inlineStr"/>
+      <c r="AC152" t="inlineStr">
+        <is>
+          <t>NPM12304</t>
+        </is>
+      </c>
       <c r="AD152" t="inlineStr"/>
+      <c r="AE152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -21366,8 +22127,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC153" t="inlineStr"/>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>NPM12305</t>
+        </is>
+      </c>
       <c r="AD153" t="inlineStr"/>
+      <c r="AE153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -21514,8 +22280,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký trái phiếu nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC154" t="inlineStr"/>
+      <c r="AC154" t="inlineStr">
+        <is>
+          <t>NPM12306</t>
+        </is>
+      </c>
       <c r="AD154" t="inlineStr"/>
+      <c r="AE154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -21658,8 +22429,13 @@
 Đề nghị các TVLK thông báo đầy đủ, chi tiết nội dung của thông báo này đến từng nhà đầu tư lưu ký chứng khoán nêu trên tại TVLK chậm nhất trong vòng 03 ngày làm việc kể từ ngày ghi trên thông báo của VSDC./.</t>
         </is>
       </c>
-      <c r="AC155" t="inlineStr"/>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>GEG12403</t>
+        </is>
+      </c>
       <c r="AD155" t="inlineStr"/>
+      <c r="AE155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -21767,8 +22543,13 @@
 Công ty Cổ phần Đệ Tam và các tổ chức, cá nhân tham gia vào quá trình lập sồ sơ, tài liệu điều chỉnh thông tin số lượng cổ phiếu đăng ký phải hoàn toàn chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2029/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC156" t="inlineStr"/>
+      <c r="AC156" t="inlineStr">
+        <is>
+          <t>DTA</t>
+        </is>
+      </c>
       <c r="AD156" t="inlineStr"/>
+      <c r="AE156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -21840,6 +22621,7 @@
       </c>
       <c r="AC157" t="inlineStr"/>
       <c r="AD157" t="inlineStr"/>
+      <c r="AE157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -21945,6 +22727,7 @@
       </c>
       <c r="AC158" t="inlineStr"/>
       <c r="AD158" t="inlineStr"/>
+      <c r="AE158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -22050,6 +22833,7 @@
       </c>
       <c r="AC159" t="inlineStr"/>
       <c r="AD159" t="inlineStr"/>
+      <c r="AE159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -22179,6 +22963,7 @@
       </c>
       <c r="AC160" t="inlineStr"/>
       <c r="AD160" t="inlineStr"/>
+      <c r="AE160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -22322,6 +23107,7 @@
       </c>
       <c r="AC161" t="inlineStr"/>
       <c r="AD161" t="inlineStr"/>
+      <c r="AE161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -22461,6 +23247,7 @@
       </c>
       <c r="AC162" t="inlineStr"/>
       <c r="AD162" t="inlineStr"/>
+      <c r="AE162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -22605,6 +23392,7 @@
       </c>
       <c r="AC163" t="inlineStr"/>
       <c r="AD163" t="inlineStr"/>
+      <c r="AE163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -22761,6 +23549,7 @@
       </c>
       <c r="AC164" t="inlineStr"/>
       <c r="AD164" t="inlineStr"/>
+      <c r="AE164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -22905,6 +23694,7 @@
       </c>
       <c r="AC165" t="inlineStr"/>
       <c r="AD165" t="inlineStr"/>
+      <c r="AE165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -23049,6 +23839,7 @@
       </c>
       <c r="AC166" t="inlineStr"/>
       <c r="AD166" t="inlineStr"/>
+      <c r="AE166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -23193,6 +23984,7 @@
       </c>
       <c r="AC167" t="inlineStr"/>
       <c r="AD167" t="inlineStr"/>
+      <c r="AE167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -23290,6 +24082,7 @@
       </c>
       <c r="AC168" t="inlineStr"/>
       <c r="AD168" t="inlineStr"/>
+      <c r="AE168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -23438,6 +24231,7 @@
       </c>
       <c r="AC169" t="inlineStr"/>
       <c r="AD169" t="inlineStr"/>
+      <c r="AE169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -23586,6 +24380,7 @@
       </c>
       <c r="AC170" t="inlineStr"/>
       <c r="AD170" t="inlineStr"/>
+      <c r="AE170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -23701,6 +24496,7 @@
       </c>
       <c r="AC171" t="inlineStr"/>
       <c r="AD171" t="inlineStr"/>
+      <c r="AE171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -23845,6 +24641,7 @@
       </c>
       <c r="AC172" t="inlineStr"/>
       <c r="AD172" t="inlineStr"/>
+      <c r="AE172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -23954,6 +24751,7 @@
       </c>
       <c r="AC173" t="inlineStr"/>
       <c r="AD173" t="inlineStr"/>
+      <c r="AE173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -24097,6 +24895,7 @@
       </c>
       <c r="AC174" t="inlineStr"/>
       <c r="AD174" t="inlineStr"/>
+      <c r="AE174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -24259,6 +25058,7 @@
       </c>
       <c r="AC175" t="inlineStr"/>
       <c r="AD175" t="inlineStr"/>
+      <c r="AE175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -24408,6 +25208,7 @@
       </c>
       <c r="AC176" t="inlineStr"/>
       <c r="AD176" t="inlineStr"/>
+      <c r="AE176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -24552,6 +25353,7 @@
       </c>
       <c r="AC177" t="inlineStr"/>
       <c r="AD177" t="inlineStr"/>
+      <c r="AE177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -24696,6 +25498,7 @@
       </c>
       <c r="AC178" t="inlineStr"/>
       <c r="AD178" t="inlineStr"/>
+      <c r="AE178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -24835,6 +25638,7 @@
       </c>
       <c r="AC179" t="inlineStr"/>
       <c r="AD179" t="inlineStr"/>
+      <c r="AE179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -24974,6 +25778,7 @@
       </c>
       <c r="AC180" t="inlineStr"/>
       <c r="AD180" t="inlineStr"/>
+      <c r="AE180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -25133,6 +25938,7 @@
       </c>
       <c r="AC181" t="inlineStr"/>
       <c r="AD181" t="inlineStr"/>
+      <c r="AE181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -25280,6 +26086,7 @@
       </c>
       <c r="AC182" t="inlineStr"/>
       <c r="AD182" t="inlineStr"/>
+      <c r="AE182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -25437,6 +26244,7 @@
       </c>
       <c r="AC183" t="inlineStr"/>
       <c r="AD183" t="inlineStr"/>
+      <c r="AE183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -25598,6 +26406,7 @@
       </c>
       <c r="AC184" t="inlineStr"/>
       <c r="AD184" t="inlineStr"/>
+      <c r="AE184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -25734,6 +26543,7 @@
       </c>
       <c r="AC185" t="inlineStr"/>
       <c r="AD185" t="inlineStr"/>
+      <c r="AE185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -25884,6 +26694,7 @@
       </c>
       <c r="AC186" t="inlineStr"/>
       <c r="AD186" t="inlineStr"/>
+      <c r="AE186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -26028,6 +26839,7 @@
       </c>
       <c r="AC187" t="inlineStr"/>
       <c r="AD187" t="inlineStr"/>
+      <c r="AE187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -26092,6 +26904,7 @@
       <c r="AB188" t="inlineStr"/>
       <c r="AC188" t="inlineStr"/>
       <c r="AD188" t="inlineStr"/>
+      <c r="AE188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -26156,6 +26969,7 @@
       <c r="AB189" t="inlineStr"/>
       <c r="AC189" t="inlineStr"/>
       <c r="AD189" t="inlineStr"/>
+      <c r="AE189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -26314,6 +27128,7 @@
       </c>
       <c r="AC190" t="inlineStr"/>
       <c r="AD190" t="inlineStr"/>
+      <c r="AE190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -26474,6 +27289,7 @@
       </c>
       <c r="AC191" t="inlineStr"/>
       <c r="AD191" t="inlineStr"/>
+      <c r="AE191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -26620,6 +27436,7 @@
       </c>
       <c r="AC192" t="inlineStr"/>
       <c r="AD192" t="inlineStr"/>
+      <c r="AE192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -26766,6 +27583,7 @@
       </c>
       <c r="AC193" t="inlineStr"/>
       <c r="AD193" t="inlineStr"/>
+      <c r="AE193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -26881,6 +27699,7 @@
       </c>
       <c r="AC194" t="inlineStr"/>
       <c r="AD194" t="inlineStr"/>
+      <c r="AE194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -27039,6 +27858,7 @@
       </c>
       <c r="AC195" t="inlineStr"/>
       <c r="AD195" t="inlineStr"/>
+      <c r="AE195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -27183,6 +28003,7 @@
       </c>
       <c r="AC196" t="inlineStr"/>
       <c r="AD196" t="inlineStr"/>
+      <c r="AE196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -27317,6 +28138,7 @@
       </c>
       <c r="AC197" t="inlineStr"/>
       <c r="AD197" t="inlineStr"/>
+      <c r="AE197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -27464,6 +28286,7 @@
       </c>
       <c r="AC198" t="inlineStr"/>
       <c r="AD198" t="inlineStr"/>
+      <c r="AE198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -27578,6 +28401,7 @@
       </c>
       <c r="AC199" t="inlineStr"/>
       <c r="AD199" t="inlineStr"/>
+      <c r="AE199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -27714,6 +28538,7 @@
       </c>
       <c r="AC200" t="inlineStr"/>
       <c r="AD200" t="inlineStr"/>
+      <c r="AE200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -27850,6 +28675,7 @@
       </c>
       <c r="AC201" t="inlineStr"/>
       <c r="AD201" t="inlineStr"/>
+      <c r="AE201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -27914,6 +28740,7 @@
       <c r="AB202" t="inlineStr"/>
       <c r="AC202" t="inlineStr"/>
       <c r="AD202" t="inlineStr"/>
+      <c r="AE202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -28080,6 +28907,7 @@
       </c>
       <c r="AC203" t="inlineStr"/>
       <c r="AD203" t="inlineStr"/>
+      <c r="AE203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -28224,6 +29052,7 @@
       </c>
       <c r="AC204" t="inlineStr"/>
       <c r="AD204" t="inlineStr"/>
+      <c r="AE204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -28295,6 +29124,7 @@
       </c>
       <c r="AC205" t="inlineStr"/>
       <c r="AD205" t="inlineStr"/>
+      <c r="AE205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -28386,12 +29216,13 @@
 CÔNG TY CỔ PHẦN JANUS GROUP và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu điều chỉnh thông tin tên TCĐKCK phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024.</t>
         </is>
       </c>
-      <c r="AC206" t="inlineStr">
+      <c r="AC206" t="inlineStr"/>
+      <c r="AD206" t="inlineStr">
         <is>
           <t>TCO</t>
         </is>
       </c>
-      <c r="AD206" t="inlineStr"/>
+      <c r="AE206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -28500,7 +29331,8 @@
       <c r="AA207" t="inlineStr"/>
       <c r="AB207" t="inlineStr"/>
       <c r="AC207" t="inlineStr"/>
-      <c r="AD207" t="inlineStr">
+      <c r="AD207" t="inlineStr"/>
+      <c r="AE207" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -28601,7 +29433,8 @@
       <c r="AA208" t="inlineStr"/>
       <c r="AB208" t="inlineStr"/>
       <c r="AC208" t="inlineStr"/>
-      <c r="AD208" t="inlineStr">
+      <c r="AD208" t="inlineStr"/>
+      <c r="AE208" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -28702,7 +29535,8 @@
       <c r="AA209" t="inlineStr"/>
       <c r="AB209" t="inlineStr"/>
       <c r="AC209" t="inlineStr"/>
-      <c r="AD209" t="inlineStr">
+      <c r="AD209" t="inlineStr"/>
+      <c r="AE209" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -28819,7 +29653,8 @@
       <c r="AA210" t="inlineStr"/>
       <c r="AB210" t="inlineStr"/>
       <c r="AC210" t="inlineStr"/>
-      <c r="AD210" t="inlineStr">
+      <c r="AD210" t="inlineStr"/>
+      <c r="AE210" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -28927,7 +29762,8 @@
       <c r="AA211" t="inlineStr"/>
       <c r="AB211" t="inlineStr"/>
       <c r="AC211" t="inlineStr"/>
-      <c r="AD211" t="inlineStr">
+      <c r="AD211" t="inlineStr"/>
+      <c r="AE211" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29035,7 +29871,8 @@
       <c r="AA212" t="inlineStr"/>
       <c r="AB212" t="inlineStr"/>
       <c r="AC212" t="inlineStr"/>
-      <c r="AD212" t="inlineStr">
+      <c r="AD212" t="inlineStr"/>
+      <c r="AE212" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29143,7 +29980,8 @@
       <c r="AA213" t="inlineStr"/>
       <c r="AB213" t="inlineStr"/>
       <c r="AC213" t="inlineStr"/>
-      <c r="AD213" t="inlineStr">
+      <c r="AD213" t="inlineStr"/>
+      <c r="AE213" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29258,7 +30096,8 @@
       <c r="AA214" t="inlineStr"/>
       <c r="AB214" t="inlineStr"/>
       <c r="AC214" t="inlineStr"/>
-      <c r="AD214" t="inlineStr">
+      <c r="AD214" t="inlineStr"/>
+      <c r="AE214" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29346,7 +30185,8 @@
       <c r="AA215" t="inlineStr"/>
       <c r="AB215" t="inlineStr"/>
       <c r="AC215" t="inlineStr"/>
-      <c r="AD215" t="inlineStr">
+      <c r="AD215" t="inlineStr"/>
+      <c r="AE215" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29434,7 +30274,8 @@
       <c r="AA216" t="inlineStr"/>
       <c r="AB216" t="inlineStr"/>
       <c r="AC216" t="inlineStr"/>
-      <c r="AD216" t="inlineStr">
+      <c r="AD216" t="inlineStr"/>
+      <c r="AE216" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29522,7 +30363,8 @@
       <c r="AA217" t="inlineStr"/>
       <c r="AB217" t="inlineStr"/>
       <c r="AC217" t="inlineStr"/>
-      <c r="AD217" t="inlineStr">
+      <c r="AD217" t="inlineStr"/>
+      <c r="AE217" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29610,7 +30452,8 @@
       <c r="AA218" t="inlineStr"/>
       <c r="AB218" t="inlineStr"/>
       <c r="AC218" t="inlineStr"/>
-      <c r="AD218" t="inlineStr">
+      <c r="AD218" t="inlineStr"/>
+      <c r="AE218" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29698,7 +30541,8 @@
       <c r="AA219" t="inlineStr"/>
       <c r="AB219" t="inlineStr"/>
       <c r="AC219" t="inlineStr"/>
-      <c r="AD219" t="inlineStr">
+      <c r="AD219" t="inlineStr"/>
+      <c r="AE219" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29794,7 +30638,8 @@
       <c r="AA220" t="inlineStr"/>
       <c r="AB220" t="inlineStr"/>
       <c r="AC220" t="inlineStr"/>
-      <c r="AD220" t="inlineStr">
+      <c r="AD220" t="inlineStr"/>
+      <c r="AE220" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -29904,7 +30749,8 @@
       <c r="AA221" t="inlineStr"/>
       <c r="AB221" t="inlineStr"/>
       <c r="AC221" t="inlineStr"/>
-      <c r="AD221" t="inlineStr">
+      <c r="AD221" t="inlineStr"/>
+      <c r="AE221" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30024,7 +30870,8 @@
       <c r="AA222" t="inlineStr"/>
       <c r="AB222" t="inlineStr"/>
       <c r="AC222" t="inlineStr"/>
-      <c r="AD222" t="inlineStr">
+      <c r="AD222" t="inlineStr"/>
+      <c r="AE222" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30149,7 +30996,8 @@
       <c r="AA223" t="inlineStr"/>
       <c r="AB223" t="inlineStr"/>
       <c r="AC223" t="inlineStr"/>
-      <c r="AD223" t="inlineStr">
+      <c r="AD223" t="inlineStr"/>
+      <c r="AE223" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30229,7 +31077,8 @@
       <c r="AA224" t="inlineStr"/>
       <c r="AB224" t="inlineStr"/>
       <c r="AC224" t="inlineStr"/>
-      <c r="AD224" t="inlineStr">
+      <c r="AD224" t="inlineStr"/>
+      <c r="AE224" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30293,7 +31142,8 @@
       <c r="AA225" t="inlineStr"/>
       <c r="AB225" t="inlineStr"/>
       <c r="AC225" t="inlineStr"/>
-      <c r="AD225" t="inlineStr">
+      <c r="AD225" t="inlineStr"/>
+      <c r="AE225" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30377,7 +31227,8 @@
       <c r="AA226" t="inlineStr"/>
       <c r="AB226" t="inlineStr"/>
       <c r="AC226" t="inlineStr"/>
-      <c r="AD226" t="inlineStr">
+      <c r="AD226" t="inlineStr"/>
+      <c r="AE226" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30461,7 +31312,8 @@
       <c r="AA227" t="inlineStr"/>
       <c r="AB227" t="inlineStr"/>
       <c r="AC227" t="inlineStr"/>
-      <c r="AD227" t="inlineStr">
+      <c r="AD227" t="inlineStr"/>
+      <c r="AE227" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30545,7 +31397,8 @@
       <c r="AA228" t="inlineStr"/>
       <c r="AB228" t="inlineStr"/>
       <c r="AC228" t="inlineStr"/>
-      <c r="AD228" t="inlineStr">
+      <c r="AD228" t="inlineStr"/>
+      <c r="AE228" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30609,7 +31462,8 @@
       <c r="AA229" t="inlineStr"/>
       <c r="AB229" t="inlineStr"/>
       <c r="AC229" t="inlineStr"/>
-      <c r="AD229" t="inlineStr">
+      <c r="AD229" t="inlineStr"/>
+      <c r="AE229" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30718,7 +31572,8 @@
       <c r="AA230" t="inlineStr"/>
       <c r="AB230" t="inlineStr"/>
       <c r="AC230" t="inlineStr"/>
-      <c r="AD230" t="inlineStr">
+      <c r="AD230" t="inlineStr"/>
+      <c r="AE230" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30832,7 +31687,8 @@
       <c r="AA231" t="inlineStr"/>
       <c r="AB231" t="inlineStr"/>
       <c r="AC231" t="inlineStr"/>
-      <c r="AD231" t="inlineStr">
+      <c r="AD231" t="inlineStr"/>
+      <c r="AE231" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -30946,7 +31802,8 @@
       <c r="AA232" t="inlineStr"/>
       <c r="AB232" t="inlineStr"/>
       <c r="AC232" t="inlineStr"/>
-      <c r="AD232" t="inlineStr">
+      <c r="AD232" t="inlineStr"/>
+      <c r="AE232" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31054,7 +31911,8 @@
       <c r="AA233" t="inlineStr"/>
       <c r="AB233" t="inlineStr"/>
       <c r="AC233" t="inlineStr"/>
-      <c r="AD233" t="inlineStr">
+      <c r="AD233" t="inlineStr"/>
+      <c r="AE233" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31159,7 +32017,8 @@
       <c r="AA234" t="inlineStr"/>
       <c r="AB234" t="inlineStr"/>
       <c r="AC234" t="inlineStr"/>
-      <c r="AD234" t="inlineStr">
+      <c r="AD234" t="inlineStr"/>
+      <c r="AE234" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31264,7 +32123,8 @@
       <c r="AA235" t="inlineStr"/>
       <c r="AB235" t="inlineStr"/>
       <c r="AC235" t="inlineStr"/>
-      <c r="AD235" t="inlineStr">
+      <c r="AD235" t="inlineStr"/>
+      <c r="AE235" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31378,7 +32238,8 @@
       <c r="AA236" t="inlineStr"/>
       <c r="AB236" t="inlineStr"/>
       <c r="AC236" t="inlineStr"/>
-      <c r="AD236" t="inlineStr">
+      <c r="AD236" t="inlineStr"/>
+      <c r="AE236" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31442,7 +32303,8 @@
       <c r="AA237" t="inlineStr"/>
       <c r="AB237" t="inlineStr"/>
       <c r="AC237" t="inlineStr"/>
-      <c r="AD237" t="inlineStr">
+      <c r="AD237" t="inlineStr"/>
+      <c r="AE237" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31545,7 +32407,8 @@
       <c r="AA238" t="inlineStr"/>
       <c r="AB238" t="inlineStr"/>
       <c r="AC238" t="inlineStr"/>
-      <c r="AD238" t="inlineStr">
+      <c r="AD238" t="inlineStr"/>
+      <c r="AE238" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31659,7 +32522,8 @@
       <c r="AA239" t="inlineStr"/>
       <c r="AB239" t="inlineStr"/>
       <c r="AC239" t="inlineStr"/>
-      <c r="AD239" t="inlineStr">
+      <c r="AD239" t="inlineStr"/>
+      <c r="AE239" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31773,7 +32637,8 @@
       <c r="AA240" t="inlineStr"/>
       <c r="AB240" t="inlineStr"/>
       <c r="AC240" t="inlineStr"/>
-      <c r="AD240" t="inlineStr">
+      <c r="AD240" t="inlineStr"/>
+      <c r="AE240" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31887,7 +32752,8 @@
       <c r="AA241" t="inlineStr"/>
       <c r="AB241" t="inlineStr"/>
       <c r="AC241" t="inlineStr"/>
-      <c r="AD241" t="inlineStr">
+      <c r="AD241" t="inlineStr"/>
+      <c r="AE241" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -31995,7 +32861,8 @@
       <c r="AA242" t="inlineStr"/>
       <c r="AB242" t="inlineStr"/>
       <c r="AC242" t="inlineStr"/>
-      <c r="AD242" t="inlineStr">
+      <c r="AD242" t="inlineStr"/>
+      <c r="AE242" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32059,7 +32926,8 @@
       <c r="AA243" t="inlineStr"/>
       <c r="AB243" t="inlineStr"/>
       <c r="AC243" t="inlineStr"/>
-      <c r="AD243" t="inlineStr">
+      <c r="AD243" t="inlineStr"/>
+      <c r="AE243" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32147,7 +33015,8 @@
       <c r="AA244" t="inlineStr"/>
       <c r="AB244" t="inlineStr"/>
       <c r="AC244" t="inlineStr"/>
-      <c r="AD244" t="inlineStr">
+      <c r="AD244" t="inlineStr"/>
+      <c r="AE244" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32235,7 +33104,8 @@
       <c r="AA245" t="inlineStr"/>
       <c r="AB245" t="inlineStr"/>
       <c r="AC245" t="inlineStr"/>
-      <c r="AD245" t="inlineStr">
+      <c r="AD245" t="inlineStr"/>
+      <c r="AE245" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32299,7 +33169,8 @@
       <c r="AA246" t="inlineStr"/>
       <c r="AB246" t="inlineStr"/>
       <c r="AC246" t="inlineStr"/>
-      <c r="AD246" t="inlineStr">
+      <c r="AD246" t="inlineStr"/>
+      <c r="AE246" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32431,7 +33302,8 @@
       <c r="AA247" t="inlineStr"/>
       <c r="AB247" t="inlineStr"/>
       <c r="AC247" t="inlineStr"/>
-      <c r="AD247" t="inlineStr">
+      <c r="AD247" t="inlineStr"/>
+      <c r="AE247" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32543,7 +33415,8 @@
       <c r="AA248" t="inlineStr"/>
       <c r="AB248" t="inlineStr"/>
       <c r="AC248" t="inlineStr"/>
-      <c r="AD248" t="inlineStr">
+      <c r="AD248" t="inlineStr"/>
+      <c r="AE248" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32636,7 +33509,8 @@
       <c r="AA249" t="inlineStr"/>
       <c r="AB249" t="inlineStr"/>
       <c r="AC249" t="inlineStr"/>
-      <c r="AD249" t="inlineStr">
+      <c r="AD249" t="inlineStr"/>
+      <c r="AE249" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32729,7 +33603,8 @@
       <c r="AA250" t="inlineStr"/>
       <c r="AB250" t="inlineStr"/>
       <c r="AC250" t="inlineStr"/>
-      <c r="AD250" t="inlineStr">
+      <c r="AD250" t="inlineStr"/>
+      <c r="AE250" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32822,7 +33697,8 @@
       <c r="AA251" t="inlineStr"/>
       <c r="AB251" t="inlineStr"/>
       <c r="AC251" t="inlineStr"/>
-      <c r="AD251" t="inlineStr">
+      <c r="AD251" t="inlineStr"/>
+      <c r="AE251" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -32915,7 +33791,8 @@
       <c r="AA252" t="inlineStr"/>
       <c r="AB252" t="inlineStr"/>
       <c r="AC252" t="inlineStr"/>
-      <c r="AD252" t="inlineStr">
+      <c r="AD252" t="inlineStr"/>
+      <c r="AE252" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33008,7 +33885,8 @@
       <c r="AA253" t="inlineStr"/>
       <c r="AB253" t="inlineStr"/>
       <c r="AC253" t="inlineStr"/>
-      <c r="AD253" t="inlineStr">
+      <c r="AD253" t="inlineStr"/>
+      <c r="AE253" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33101,7 +33979,8 @@
       <c r="AA254" t="inlineStr"/>
       <c r="AB254" t="inlineStr"/>
       <c r="AC254" t="inlineStr"/>
-      <c r="AD254" t="inlineStr">
+      <c r="AD254" t="inlineStr"/>
+      <c r="AE254" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33194,7 +34073,8 @@
       <c r="AA255" t="inlineStr"/>
       <c r="AB255" t="inlineStr"/>
       <c r="AC255" t="inlineStr"/>
-      <c r="AD255" t="inlineStr">
+      <c r="AD255" t="inlineStr"/>
+      <c r="AE255" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33287,7 +34167,8 @@
       <c r="AA256" t="inlineStr"/>
       <c r="AB256" t="inlineStr"/>
       <c r="AC256" t="inlineStr"/>
-      <c r="AD256" t="inlineStr">
+      <c r="AD256" t="inlineStr"/>
+      <c r="AE256" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33380,7 +34261,8 @@
       <c r="AA257" t="inlineStr"/>
       <c r="AB257" t="inlineStr"/>
       <c r="AC257" t="inlineStr"/>
-      <c r="AD257" t="inlineStr">
+      <c r="AD257" t="inlineStr"/>
+      <c r="AE257" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33473,7 +34355,8 @@
       <c r="AA258" t="inlineStr"/>
       <c r="AB258" t="inlineStr"/>
       <c r="AC258" t="inlineStr"/>
-      <c r="AD258" t="inlineStr">
+      <c r="AD258" t="inlineStr"/>
+      <c r="AE258" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33590,7 +34473,8 @@
       <c r="AA259" t="inlineStr"/>
       <c r="AB259" t="inlineStr"/>
       <c r="AC259" t="inlineStr"/>
-      <c r="AD259" t="inlineStr">
+      <c r="AD259" t="inlineStr"/>
+      <c r="AE259" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33704,7 +34588,8 @@
       <c r="AA260" t="inlineStr"/>
       <c r="AB260" t="inlineStr"/>
       <c r="AC260" t="inlineStr"/>
-      <c r="AD260" t="inlineStr">
+      <c r="AD260" t="inlineStr"/>
+      <c r="AE260" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33828,7 +34713,8 @@
       <c r="AA261" t="inlineStr"/>
       <c r="AB261" t="inlineStr"/>
       <c r="AC261" t="inlineStr"/>
-      <c r="AD261" t="inlineStr">
+      <c r="AD261" t="inlineStr"/>
+      <c r="AE261" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -33945,7 +34831,8 @@
       <c r="AA262" t="inlineStr"/>
       <c r="AB262" t="inlineStr"/>
       <c r="AC262" t="inlineStr"/>
-      <c r="AD262" t="inlineStr">
+      <c r="AD262" t="inlineStr"/>
+      <c r="AE262" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34065,7 +34952,8 @@
       <c r="AA263" t="inlineStr"/>
       <c r="AB263" t="inlineStr"/>
       <c r="AC263" t="inlineStr"/>
-      <c r="AD263" t="inlineStr">
+      <c r="AD263" t="inlineStr"/>
+      <c r="AE263" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34185,7 +35073,8 @@
       <c r="AA264" t="inlineStr"/>
       <c r="AB264" t="inlineStr"/>
       <c r="AC264" t="inlineStr"/>
-      <c r="AD264" t="inlineStr">
+      <c r="AD264" t="inlineStr"/>
+      <c r="AE264" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34273,7 +35162,8 @@
       <c r="AA265" t="inlineStr"/>
       <c r="AB265" t="inlineStr"/>
       <c r="AC265" t="inlineStr"/>
-      <c r="AD265" t="inlineStr">
+      <c r="AD265" t="inlineStr"/>
+      <c r="AE265" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34361,7 +35251,8 @@
       <c r="AA266" t="inlineStr"/>
       <c r="AB266" t="inlineStr"/>
       <c r="AC266" t="inlineStr"/>
-      <c r="AD266" t="inlineStr">
+      <c r="AD266" t="inlineStr"/>
+      <c r="AE266" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34454,7 +35345,8 @@
       <c r="AA267" t="inlineStr"/>
       <c r="AB267" t="inlineStr"/>
       <c r="AC267" t="inlineStr"/>
-      <c r="AD267" t="inlineStr">
+      <c r="AD267" t="inlineStr"/>
+      <c r="AE267" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34547,7 +35439,8 @@
       <c r="AA268" t="inlineStr"/>
       <c r="AB268" t="inlineStr"/>
       <c r="AC268" t="inlineStr"/>
-      <c r="AD268" t="inlineStr">
+      <c r="AD268" t="inlineStr"/>
+      <c r="AE268" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34640,7 +35533,8 @@
       <c r="AA269" t="inlineStr"/>
       <c r="AB269" t="inlineStr"/>
       <c r="AC269" t="inlineStr"/>
-      <c r="AD269" t="inlineStr">
+      <c r="AD269" t="inlineStr"/>
+      <c r="AE269" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34733,7 +35627,8 @@
       <c r="AA270" t="inlineStr"/>
       <c r="AB270" t="inlineStr"/>
       <c r="AC270" t="inlineStr"/>
-      <c r="AD270" t="inlineStr">
+      <c r="AD270" t="inlineStr"/>
+      <c r="AE270" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34826,7 +35721,8 @@
       <c r="AA271" t="inlineStr"/>
       <c r="AB271" t="inlineStr"/>
       <c r="AC271" t="inlineStr"/>
-      <c r="AD271" t="inlineStr">
+      <c r="AD271" t="inlineStr"/>
+      <c r="AE271" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -34919,7 +35815,8 @@
       <c r="AA272" t="inlineStr"/>
       <c r="AB272" t="inlineStr"/>
       <c r="AC272" t="inlineStr"/>
-      <c r="AD272" t="inlineStr">
+      <c r="AD272" t="inlineStr"/>
+      <c r="AE272" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35012,7 +35909,8 @@
       <c r="AA273" t="inlineStr"/>
       <c r="AB273" t="inlineStr"/>
       <c r="AC273" t="inlineStr"/>
-      <c r="AD273" t="inlineStr">
+      <c r="AD273" t="inlineStr"/>
+      <c r="AE273" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35105,7 +36003,8 @@
       <c r="AA274" t="inlineStr"/>
       <c r="AB274" t="inlineStr"/>
       <c r="AC274" t="inlineStr"/>
-      <c r="AD274" t="inlineStr">
+      <c r="AD274" t="inlineStr"/>
+      <c r="AE274" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35217,7 +36116,8 @@
       <c r="AA275" t="inlineStr"/>
       <c r="AB275" t="inlineStr"/>
       <c r="AC275" t="inlineStr"/>
-      <c r="AD275" t="inlineStr">
+      <c r="AD275" t="inlineStr"/>
+      <c r="AE275" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35310,7 +36210,8 @@
       <c r="AA276" t="inlineStr"/>
       <c r="AB276" t="inlineStr"/>
       <c r="AC276" t="inlineStr"/>
-      <c r="AD276" t="inlineStr">
+      <c r="AD276" t="inlineStr"/>
+      <c r="AE276" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35378,7 +36279,8 @@
       <c r="AA277" t="inlineStr"/>
       <c r="AB277" t="inlineStr"/>
       <c r="AC277" t="inlineStr"/>
-      <c r="AD277" t="inlineStr">
+      <c r="AD277" t="inlineStr"/>
+      <c r="AE277" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35471,7 +36373,8 @@
       <c r="AA278" t="inlineStr"/>
       <c r="AB278" t="inlineStr"/>
       <c r="AC278" t="inlineStr"/>
-      <c r="AD278" t="inlineStr">
+      <c r="AD278" t="inlineStr"/>
+      <c r="AE278" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35564,7 +36467,8 @@
       <c r="AA279" t="inlineStr"/>
       <c r="AB279" t="inlineStr"/>
       <c r="AC279" t="inlineStr"/>
-      <c r="AD279" t="inlineStr">
+      <c r="AD279" t="inlineStr"/>
+      <c r="AE279" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35657,7 +36561,8 @@
       <c r="AA280" t="inlineStr"/>
       <c r="AB280" t="inlineStr"/>
       <c r="AC280" t="inlineStr"/>
-      <c r="AD280" t="inlineStr">
+      <c r="AD280" t="inlineStr"/>
+      <c r="AE280" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35750,7 +36655,8 @@
       <c r="AA281" t="inlineStr"/>
       <c r="AB281" t="inlineStr"/>
       <c r="AC281" t="inlineStr"/>
-      <c r="AD281" t="inlineStr">
+      <c r="AD281" t="inlineStr"/>
+      <c r="AE281" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35843,7 +36749,8 @@
       <c r="AA282" t="inlineStr"/>
       <c r="AB282" t="inlineStr"/>
       <c r="AC282" t="inlineStr"/>
-      <c r="AD282" t="inlineStr">
+      <c r="AD282" t="inlineStr"/>
+      <c r="AE282" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -35936,7 +36843,8 @@
       <c r="AA283" t="inlineStr"/>
       <c r="AB283" t="inlineStr"/>
       <c r="AC283" t="inlineStr"/>
-      <c r="AD283" t="inlineStr">
+      <c r="AD283" t="inlineStr"/>
+      <c r="AE283" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36029,7 +36937,8 @@
       <c r="AA284" t="inlineStr"/>
       <c r="AB284" t="inlineStr"/>
       <c r="AC284" t="inlineStr"/>
-      <c r="AD284" t="inlineStr">
+      <c r="AD284" t="inlineStr"/>
+      <c r="AE284" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36143,7 +37052,8 @@
       <c r="AA285" t="inlineStr"/>
       <c r="AB285" t="inlineStr"/>
       <c r="AC285" t="inlineStr"/>
-      <c r="AD285" t="inlineStr">
+      <c r="AD285" t="inlineStr"/>
+      <c r="AE285" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36255,7 +37165,8 @@
       <c r="AA286" t="inlineStr"/>
       <c r="AB286" t="inlineStr"/>
       <c r="AC286" t="inlineStr"/>
-      <c r="AD286" t="inlineStr">
+      <c r="AD286" t="inlineStr"/>
+      <c r="AE286" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36367,7 +37278,8 @@
       <c r="AA287" t="inlineStr"/>
       <c r="AB287" t="inlineStr"/>
       <c r="AC287" t="inlineStr"/>
-      <c r="AD287" t="inlineStr">
+      <c r="AD287" t="inlineStr"/>
+      <c r="AE287" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36480,7 +37392,8 @@
       <c r="AA288" t="inlineStr"/>
       <c r="AB288" t="inlineStr"/>
       <c r="AC288" t="inlineStr"/>
-      <c r="AD288" t="inlineStr">
+      <c r="AD288" t="inlineStr"/>
+      <c r="AE288" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36588,7 +37501,8 @@
       <c r="AA289" t="inlineStr"/>
       <c r="AB289" t="inlineStr"/>
       <c r="AC289" t="inlineStr"/>
-      <c r="AD289" t="inlineStr">
+      <c r="AD289" t="inlineStr"/>
+      <c r="AE289" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36702,7 +37616,8 @@
       <c r="AA290" t="inlineStr"/>
       <c r="AB290" t="inlineStr"/>
       <c r="AC290" t="inlineStr"/>
-      <c r="AD290" t="inlineStr">
+      <c r="AD290" t="inlineStr"/>
+      <c r="AE290" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36814,7 +37729,8 @@
       <c r="AA291" t="inlineStr"/>
       <c r="AB291" t="inlineStr"/>
       <c r="AC291" t="inlineStr"/>
-      <c r="AD291" t="inlineStr">
+      <c r="AD291" t="inlineStr"/>
+      <c r="AE291" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -36928,7 +37844,8 @@
       <c r="AA292" t="inlineStr"/>
       <c r="AB292" t="inlineStr"/>
       <c r="AC292" t="inlineStr"/>
-      <c r="AD292" t="inlineStr">
+      <c r="AD292" t="inlineStr"/>
+      <c r="AE292" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37042,7 +37959,8 @@
       <c r="AA293" t="inlineStr"/>
       <c r="AB293" t="inlineStr"/>
       <c r="AC293" t="inlineStr"/>
-      <c r="AD293" t="inlineStr">
+      <c r="AD293" t="inlineStr"/>
+      <c r="AE293" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37135,7 +38053,8 @@
       <c r="AA294" t="inlineStr"/>
       <c r="AB294" t="inlineStr"/>
       <c r="AC294" t="inlineStr"/>
-      <c r="AD294" t="inlineStr">
+      <c r="AD294" t="inlineStr"/>
+      <c r="AE294" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37236,7 +38155,8 @@
       <c r="AA295" t="inlineStr"/>
       <c r="AB295" t="inlineStr"/>
       <c r="AC295" t="inlineStr"/>
-      <c r="AD295" t="inlineStr">
+      <c r="AD295" t="inlineStr"/>
+      <c r="AE295" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37344,7 +38264,8 @@
       <c r="AA296" t="inlineStr"/>
       <c r="AB296" t="inlineStr"/>
       <c r="AC296" t="inlineStr"/>
-      <c r="AD296" t="inlineStr">
+      <c r="AD296" t="inlineStr"/>
+      <c r="AE296" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37461,7 +38382,8 @@
       <c r="AA297" t="inlineStr"/>
       <c r="AB297" t="inlineStr"/>
       <c r="AC297" t="inlineStr"/>
-      <c r="AD297" t="inlineStr">
+      <c r="AD297" t="inlineStr"/>
+      <c r="AE297" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37557,7 +38479,8 @@
       <c r="AA298" t="inlineStr"/>
       <c r="AB298" t="inlineStr"/>
       <c r="AC298" t="inlineStr"/>
-      <c r="AD298" t="inlineStr">
+      <c r="AD298" t="inlineStr"/>
+      <c r="AE298" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37653,7 +38576,8 @@
       <c r="AA299" t="inlineStr"/>
       <c r="AB299" t="inlineStr"/>
       <c r="AC299" t="inlineStr"/>
-      <c r="AD299" t="inlineStr">
+      <c r="AD299" t="inlineStr"/>
+      <c r="AE299" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37749,7 +38673,8 @@
       <c r="AA300" t="inlineStr"/>
       <c r="AB300" t="inlineStr"/>
       <c r="AC300" t="inlineStr"/>
-      <c r="AD300" t="inlineStr">
+      <c r="AD300" t="inlineStr"/>
+      <c r="AE300" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37845,7 +38770,8 @@
       <c r="AA301" t="inlineStr"/>
       <c r="AB301" t="inlineStr"/>
       <c r="AC301" t="inlineStr"/>
-      <c r="AD301" t="inlineStr">
+      <c r="AD301" t="inlineStr"/>
+      <c r="AE301" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -37941,7 +38867,8 @@
       <c r="AA302" t="inlineStr"/>
       <c r="AB302" t="inlineStr"/>
       <c r="AC302" t="inlineStr"/>
-      <c r="AD302" t="inlineStr">
+      <c r="AD302" t="inlineStr"/>
+      <c r="AE302" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38037,7 +38964,8 @@
       <c r="AA303" t="inlineStr"/>
       <c r="AB303" t="inlineStr"/>
       <c r="AC303" t="inlineStr"/>
-      <c r="AD303" t="inlineStr">
+      <c r="AD303" t="inlineStr"/>
+      <c r="AE303" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38133,7 +39061,8 @@
       <c r="AA304" t="inlineStr"/>
       <c r="AB304" t="inlineStr"/>
       <c r="AC304" t="inlineStr"/>
-      <c r="AD304" t="inlineStr">
+      <c r="AD304" t="inlineStr"/>
+      <c r="AE304" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38229,7 +39158,8 @@
       <c r="AA305" t="inlineStr"/>
       <c r="AB305" t="inlineStr"/>
       <c r="AC305" t="inlineStr"/>
-      <c r="AD305" t="inlineStr">
+      <c r="AD305" t="inlineStr"/>
+      <c r="AE305" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38325,7 +39255,8 @@
       <c r="AA306" t="inlineStr"/>
       <c r="AB306" t="inlineStr"/>
       <c r="AC306" t="inlineStr"/>
-      <c r="AD306" t="inlineStr">
+      <c r="AD306" t="inlineStr"/>
+      <c r="AE306" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38421,7 +39352,8 @@
       <c r="AA307" t="inlineStr"/>
       <c r="AB307" t="inlineStr"/>
       <c r="AC307" t="inlineStr"/>
-      <c r="AD307" t="inlineStr">
+      <c r="AD307" t="inlineStr"/>
+      <c r="AE307" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38517,7 +39449,8 @@
       <c r="AA308" t="inlineStr"/>
       <c r="AB308" t="inlineStr"/>
       <c r="AC308" t="inlineStr"/>
-      <c r="AD308" t="inlineStr">
+      <c r="AD308" t="inlineStr"/>
+      <c r="AE308" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38613,7 +39546,8 @@
       <c r="AA309" t="inlineStr"/>
       <c r="AB309" t="inlineStr"/>
       <c r="AC309" t="inlineStr"/>
-      <c r="AD309" t="inlineStr">
+      <c r="AD309" t="inlineStr"/>
+      <c r="AE309" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38709,7 +39643,8 @@
       <c r="AA310" t="inlineStr"/>
       <c r="AB310" t="inlineStr"/>
       <c r="AC310" t="inlineStr"/>
-      <c r="AD310" t="inlineStr">
+      <c r="AD310" t="inlineStr"/>
+      <c r="AE310" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38814,7 +39749,8 @@
       <c r="AA311" t="inlineStr"/>
       <c r="AB311" t="inlineStr"/>
       <c r="AC311" t="inlineStr"/>
-      <c r="AD311" t="inlineStr">
+      <c r="AD311" t="inlineStr"/>
+      <c r="AE311" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -38910,7 +39846,8 @@
       <c r="AA312" t="inlineStr"/>
       <c r="AB312" t="inlineStr"/>
       <c r="AC312" t="inlineStr"/>
-      <c r="AD312" t="inlineStr">
+      <c r="AD312" t="inlineStr"/>
+      <c r="AE312" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39006,7 +39943,8 @@
       <c r="AA313" t="inlineStr"/>
       <c r="AB313" t="inlineStr"/>
       <c r="AC313" t="inlineStr"/>
-      <c r="AD313" t="inlineStr">
+      <c r="AD313" t="inlineStr"/>
+      <c r="AE313" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39102,7 +40040,8 @@
       <c r="AA314" t="inlineStr"/>
       <c r="AB314" t="inlineStr"/>
       <c r="AC314" t="inlineStr"/>
-      <c r="AD314" t="inlineStr">
+      <c r="AD314" t="inlineStr"/>
+      <c r="AE314" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39198,7 +40137,8 @@
       <c r="AA315" t="inlineStr"/>
       <c r="AB315" t="inlineStr"/>
       <c r="AC315" t="inlineStr"/>
-      <c r="AD315" t="inlineStr">
+      <c r="AD315" t="inlineStr"/>
+      <c r="AE315" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39294,7 +40234,8 @@
       <c r="AA316" t="inlineStr"/>
       <c r="AB316" t="inlineStr"/>
       <c r="AC316" t="inlineStr"/>
-      <c r="AD316" t="inlineStr">
+      <c r="AD316" t="inlineStr"/>
+      <c r="AE316" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39390,7 +40331,8 @@
       <c r="AA317" t="inlineStr"/>
       <c r="AB317" t="inlineStr"/>
       <c r="AC317" t="inlineStr"/>
-      <c r="AD317" t="inlineStr">
+      <c r="AD317" t="inlineStr"/>
+      <c r="AE317" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39486,7 +40428,8 @@
       <c r="AA318" t="inlineStr"/>
       <c r="AB318" t="inlineStr"/>
       <c r="AC318" t="inlineStr"/>
-      <c r="AD318" t="inlineStr">
+      <c r="AD318" t="inlineStr"/>
+      <c r="AE318" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39582,7 +40525,8 @@
       <c r="AA319" t="inlineStr"/>
       <c r="AB319" t="inlineStr"/>
       <c r="AC319" t="inlineStr"/>
-      <c r="AD319" t="inlineStr">
+      <c r="AD319" t="inlineStr"/>
+      <c r="AE319" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39705,7 +40649,8 @@
       <c r="AA320" t="inlineStr"/>
       <c r="AB320" t="inlineStr"/>
       <c r="AC320" t="inlineStr"/>
-      <c r="AD320" t="inlineStr">
+      <c r="AD320" t="inlineStr"/>
+      <c r="AE320" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39819,7 +40764,8 @@
       <c r="AA321" t="inlineStr"/>
       <c r="AB321" t="inlineStr"/>
       <c r="AC321" t="inlineStr"/>
-      <c r="AD321" t="inlineStr">
+      <c r="AD321" t="inlineStr"/>
+      <c r="AE321" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -39933,7 +40879,8 @@
       <c r="AA322" t="inlineStr"/>
       <c r="AB322" t="inlineStr"/>
       <c r="AC322" t="inlineStr"/>
-      <c r="AD322" t="inlineStr">
+      <c r="AD322" t="inlineStr"/>
+      <c r="AE322" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40040,7 +40987,8 @@
       <c r="AA323" t="inlineStr"/>
       <c r="AB323" t="inlineStr"/>
       <c r="AC323" t="inlineStr"/>
-      <c r="AD323" t="inlineStr">
+      <c r="AD323" t="inlineStr"/>
+      <c r="AE323" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40104,7 +41052,8 @@
       <c r="AA324" t="inlineStr"/>
       <c r="AB324" t="inlineStr"/>
       <c r="AC324" t="inlineStr"/>
-      <c r="AD324" t="inlineStr">
+      <c r="AD324" t="inlineStr"/>
+      <c r="AE324" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40218,7 +41167,8 @@
       <c r="AA325" t="inlineStr"/>
       <c r="AB325" t="inlineStr"/>
       <c r="AC325" t="inlineStr"/>
-      <c r="AD325" t="inlineStr">
+      <c r="AD325" t="inlineStr"/>
+      <c r="AE325" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40311,7 +41261,8 @@
       <c r="AA326" t="inlineStr"/>
       <c r="AB326" t="inlineStr"/>
       <c r="AC326" t="inlineStr"/>
-      <c r="AD326" t="inlineStr">
+      <c r="AD326" t="inlineStr"/>
+      <c r="AE326" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40425,7 +41376,8 @@
       <c r="AA327" t="inlineStr"/>
       <c r="AB327" t="inlineStr"/>
       <c r="AC327" t="inlineStr"/>
-      <c r="AD327" t="inlineStr">
+      <c r="AD327" t="inlineStr"/>
+      <c r="AE327" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40551,7 +41503,8 @@
       <c r="AA328" t="inlineStr"/>
       <c r="AB328" t="inlineStr"/>
       <c r="AC328" t="inlineStr"/>
-      <c r="AD328" t="inlineStr">
+      <c r="AD328" t="inlineStr"/>
+      <c r="AE328" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40659,7 +41612,8 @@
       <c r="AA329" t="inlineStr"/>
       <c r="AB329" t="inlineStr"/>
       <c r="AC329" t="inlineStr"/>
-      <c r="AD329" t="inlineStr">
+      <c r="AD329" t="inlineStr"/>
+      <c r="AE329" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40776,7 +41730,8 @@
       <c r="AA330" t="inlineStr"/>
       <c r="AB330" t="inlineStr"/>
       <c r="AC330" t="inlineStr"/>
-      <c r="AD330" t="inlineStr">
+      <c r="AD330" t="inlineStr"/>
+      <c r="AE330" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40869,7 +41824,8 @@
       <c r="AA331" t="inlineStr"/>
       <c r="AB331" t="inlineStr"/>
       <c r="AC331" t="inlineStr"/>
-      <c r="AD331" t="inlineStr">
+      <c r="AD331" t="inlineStr"/>
+      <c r="AE331" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -40962,7 +41918,8 @@
       <c r="AA332" t="inlineStr"/>
       <c r="AB332" t="inlineStr"/>
       <c r="AC332" t="inlineStr"/>
-      <c r="AD332" t="inlineStr">
+      <c r="AD332" t="inlineStr"/>
+      <c r="AE332" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41055,7 +42012,8 @@
       <c r="AA333" t="inlineStr"/>
       <c r="AB333" t="inlineStr"/>
       <c r="AC333" t="inlineStr"/>
-      <c r="AD333" t="inlineStr">
+      <c r="AD333" t="inlineStr"/>
+      <c r="AE333" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41148,7 +42106,8 @@
       <c r="AA334" t="inlineStr"/>
       <c r="AB334" t="inlineStr"/>
       <c r="AC334" t="inlineStr"/>
-      <c r="AD334" t="inlineStr">
+      <c r="AD334" t="inlineStr"/>
+      <c r="AE334" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41241,7 +42200,8 @@
       <c r="AA335" t="inlineStr"/>
       <c r="AB335" t="inlineStr"/>
       <c r="AC335" t="inlineStr"/>
-      <c r="AD335" t="inlineStr">
+      <c r="AD335" t="inlineStr"/>
+      <c r="AE335" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41334,7 +42294,8 @@
       <c r="AA336" t="inlineStr"/>
       <c r="AB336" t="inlineStr"/>
       <c r="AC336" t="inlineStr"/>
-      <c r="AD336" t="inlineStr">
+      <c r="AD336" t="inlineStr"/>
+      <c r="AE336" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41427,7 +42388,8 @@
       <c r="AA337" t="inlineStr"/>
       <c r="AB337" t="inlineStr"/>
       <c r="AC337" t="inlineStr"/>
-      <c r="AD337" t="inlineStr">
+      <c r="AD337" t="inlineStr"/>
+      <c r="AE337" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41520,7 +42482,8 @@
       <c r="AA338" t="inlineStr"/>
       <c r="AB338" t="inlineStr"/>
       <c r="AC338" t="inlineStr"/>
-      <c r="AD338" t="inlineStr">
+      <c r="AD338" t="inlineStr"/>
+      <c r="AE338" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41613,7 +42576,8 @@
       <c r="AA339" t="inlineStr"/>
       <c r="AB339" t="inlineStr"/>
       <c r="AC339" t="inlineStr"/>
-      <c r="AD339" t="inlineStr">
+      <c r="AD339" t="inlineStr"/>
+      <c r="AE339" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41706,7 +42670,8 @@
       <c r="AA340" t="inlineStr"/>
       <c r="AB340" t="inlineStr"/>
       <c r="AC340" t="inlineStr"/>
-      <c r="AD340" t="inlineStr">
+      <c r="AD340" t="inlineStr"/>
+      <c r="AE340" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41799,7 +42764,8 @@
       <c r="AA341" t="inlineStr"/>
       <c r="AB341" t="inlineStr"/>
       <c r="AC341" t="inlineStr"/>
-      <c r="AD341" t="inlineStr">
+      <c r="AD341" t="inlineStr"/>
+      <c r="AE341" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41892,7 +42858,8 @@
       <c r="AA342" t="inlineStr"/>
       <c r="AB342" t="inlineStr"/>
       <c r="AC342" t="inlineStr"/>
-      <c r="AD342" t="inlineStr">
+      <c r="AD342" t="inlineStr"/>
+      <c r="AE342" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -41985,7 +42952,8 @@
       <c r="AA343" t="inlineStr"/>
       <c r="AB343" t="inlineStr"/>
       <c r="AC343" t="inlineStr"/>
-      <c r="AD343" t="inlineStr">
+      <c r="AD343" t="inlineStr"/>
+      <c r="AE343" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42078,7 +43046,8 @@
       <c r="AA344" t="inlineStr"/>
       <c r="AB344" t="inlineStr"/>
       <c r="AC344" t="inlineStr"/>
-      <c r="AD344" t="inlineStr">
+      <c r="AD344" t="inlineStr"/>
+      <c r="AE344" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42171,7 +43140,8 @@
       <c r="AA345" t="inlineStr"/>
       <c r="AB345" t="inlineStr"/>
       <c r="AC345" t="inlineStr"/>
-      <c r="AD345" t="inlineStr">
+      <c r="AD345" t="inlineStr"/>
+      <c r="AE345" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42264,7 +43234,8 @@
       <c r="AA346" t="inlineStr"/>
       <c r="AB346" t="inlineStr"/>
       <c r="AC346" t="inlineStr"/>
-      <c r="AD346" t="inlineStr">
+      <c r="AD346" t="inlineStr"/>
+      <c r="AE346" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42357,7 +43328,8 @@
       <c r="AA347" t="inlineStr"/>
       <c r="AB347" t="inlineStr"/>
       <c r="AC347" t="inlineStr"/>
-      <c r="AD347" t="inlineStr">
+      <c r="AD347" t="inlineStr"/>
+      <c r="AE347" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42450,7 +43422,8 @@
       <c r="AA348" t="inlineStr"/>
       <c r="AB348" t="inlineStr"/>
       <c r="AC348" t="inlineStr"/>
-      <c r="AD348" t="inlineStr">
+      <c r="AD348" t="inlineStr"/>
+      <c r="AE348" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42543,7 +43516,8 @@
       <c r="AA349" t="inlineStr"/>
       <c r="AB349" t="inlineStr"/>
       <c r="AC349" t="inlineStr"/>
-      <c r="AD349" t="inlineStr">
+      <c r="AD349" t="inlineStr"/>
+      <c r="AE349" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42636,7 +43610,8 @@
       <c r="AA350" t="inlineStr"/>
       <c r="AB350" t="inlineStr"/>
       <c r="AC350" t="inlineStr"/>
-      <c r="AD350" t="inlineStr">
+      <c r="AD350" t="inlineStr"/>
+      <c r="AE350" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42729,7 +43704,8 @@
       <c r="AA351" t="inlineStr"/>
       <c r="AB351" t="inlineStr"/>
       <c r="AC351" t="inlineStr"/>
-      <c r="AD351" t="inlineStr">
+      <c r="AD351" t="inlineStr"/>
+      <c r="AE351" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42822,7 +43798,8 @@
       <c r="AA352" t="inlineStr"/>
       <c r="AB352" t="inlineStr"/>
       <c r="AC352" t="inlineStr"/>
-      <c r="AD352" t="inlineStr">
+      <c r="AD352" t="inlineStr"/>
+      <c r="AE352" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -42915,7 +43892,8 @@
       <c r="AA353" t="inlineStr"/>
       <c r="AB353" t="inlineStr"/>
       <c r="AC353" t="inlineStr"/>
-      <c r="AD353" t="inlineStr">
+      <c r="AD353" t="inlineStr"/>
+      <c r="AE353" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43008,7 +43986,8 @@
       <c r="AA354" t="inlineStr"/>
       <c r="AB354" t="inlineStr"/>
       <c r="AC354" t="inlineStr"/>
-      <c r="AD354" t="inlineStr">
+      <c r="AD354" t="inlineStr"/>
+      <c r="AE354" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43101,7 +44080,8 @@
       <c r="AA355" t="inlineStr"/>
       <c r="AB355" t="inlineStr"/>
       <c r="AC355" t="inlineStr"/>
-      <c r="AD355" t="inlineStr">
+      <c r="AD355" t="inlineStr"/>
+      <c r="AE355" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43194,7 +44174,8 @@
       <c r="AA356" t="inlineStr"/>
       <c r="AB356" t="inlineStr"/>
       <c r="AC356" t="inlineStr"/>
-      <c r="AD356" t="inlineStr">
+      <c r="AD356" t="inlineStr"/>
+      <c r="AE356" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43287,7 +44268,8 @@
       <c r="AA357" t="inlineStr"/>
       <c r="AB357" t="inlineStr"/>
       <c r="AC357" t="inlineStr"/>
-      <c r="AD357" t="inlineStr">
+      <c r="AD357" t="inlineStr"/>
+      <c r="AE357" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43380,7 +44362,8 @@
       <c r="AA358" t="inlineStr"/>
       <c r="AB358" t="inlineStr"/>
       <c r="AC358" t="inlineStr"/>
-      <c r="AD358" t="inlineStr">
+      <c r="AD358" t="inlineStr"/>
+      <c r="AE358" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43473,7 +44456,8 @@
       <c r="AA359" t="inlineStr"/>
       <c r="AB359" t="inlineStr"/>
       <c r="AC359" t="inlineStr"/>
-      <c r="AD359" t="inlineStr">
+      <c r="AD359" t="inlineStr"/>
+      <c r="AE359" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43557,7 +44541,8 @@
       <c r="AA360" t="inlineStr"/>
       <c r="AB360" t="inlineStr"/>
       <c r="AC360" t="inlineStr"/>
-      <c r="AD360" t="inlineStr">
+      <c r="AD360" t="inlineStr"/>
+      <c r="AE360" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43645,7 +44630,8 @@
       <c r="AA361" t="inlineStr"/>
       <c r="AB361" t="inlineStr"/>
       <c r="AC361" t="inlineStr"/>
-      <c r="AD361" t="inlineStr">
+      <c r="AD361" t="inlineStr"/>
+      <c r="AE361" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43733,7 +44719,8 @@
       <c r="AA362" t="inlineStr"/>
       <c r="AB362" t="inlineStr"/>
       <c r="AC362" t="inlineStr"/>
-      <c r="AD362" t="inlineStr">
+      <c r="AD362" t="inlineStr"/>
+      <c r="AE362" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43821,7 +44808,8 @@
       <c r="AA363" t="inlineStr"/>
       <c r="AB363" t="inlineStr"/>
       <c r="AC363" t="inlineStr"/>
-      <c r="AD363" t="inlineStr">
+      <c r="AD363" t="inlineStr"/>
+      <c r="AE363" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -43935,7 +44923,8 @@
       <c r="AA364" t="inlineStr"/>
       <c r="AB364" t="inlineStr"/>
       <c r="AC364" t="inlineStr"/>
-      <c r="AD364" t="inlineStr">
+      <c r="AD364" t="inlineStr"/>
+      <c r="AE364" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44040,7 +45029,8 @@
       <c r="AA365" t="inlineStr"/>
       <c r="AB365" t="inlineStr"/>
       <c r="AC365" t="inlineStr"/>
-      <c r="AD365" t="inlineStr">
+      <c r="AD365" t="inlineStr"/>
+      <c r="AE365" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44124,7 +45114,8 @@
       <c r="AA366" t="inlineStr"/>
       <c r="AB366" t="inlineStr"/>
       <c r="AC366" t="inlineStr"/>
-      <c r="AD366" t="inlineStr">
+      <c r="AD366" t="inlineStr"/>
+      <c r="AE366" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44237,7 +45228,8 @@
       <c r="AA367" t="inlineStr"/>
       <c r="AB367" t="inlineStr"/>
       <c r="AC367" t="inlineStr"/>
-      <c r="AD367" t="inlineStr">
+      <c r="AD367" t="inlineStr"/>
+      <c r="AE367" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44350,7 +45342,8 @@
       <c r="AA368" t="inlineStr"/>
       <c r="AB368" t="inlineStr"/>
       <c r="AC368" t="inlineStr"/>
-      <c r="AD368" t="inlineStr">
+      <c r="AD368" t="inlineStr"/>
+      <c r="AE368" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44459,7 +45452,8 @@
       <c r="AA369" t="inlineStr"/>
       <c r="AB369" t="inlineStr"/>
       <c r="AC369" t="inlineStr"/>
-      <c r="AD369" t="inlineStr">
+      <c r="AD369" t="inlineStr"/>
+      <c r="AE369" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44559,7 +45553,8 @@
       <c r="AA370" t="inlineStr"/>
       <c r="AB370" t="inlineStr"/>
       <c r="AC370" t="inlineStr"/>
-      <c r="AD370" t="inlineStr">
+      <c r="AD370" t="inlineStr"/>
+      <c r="AE370" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44674,7 +45669,8 @@
       <c r="AA371" t="inlineStr"/>
       <c r="AB371" t="inlineStr"/>
       <c r="AC371" t="inlineStr"/>
-      <c r="AD371" t="inlineStr">
+      <c r="AD371" t="inlineStr"/>
+      <c r="AE371" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44801,7 +45797,8 @@
       <c r="AA372" t="inlineStr"/>
       <c r="AB372" t="inlineStr"/>
       <c r="AC372" t="inlineStr"/>
-      <c r="AD372" t="inlineStr">
+      <c r="AD372" t="inlineStr"/>
+      <c r="AE372" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -44909,7 +45906,8 @@
       <c r="AA373" t="inlineStr"/>
       <c r="AB373" t="inlineStr"/>
       <c r="AC373" t="inlineStr"/>
-      <c r="AD373" t="inlineStr">
+      <c r="AD373" t="inlineStr"/>
+      <c r="AE373" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45023,7 +46021,8 @@
       <c r="AA374" t="inlineStr"/>
       <c r="AB374" t="inlineStr"/>
       <c r="AC374" t="inlineStr"/>
-      <c r="AD374" t="inlineStr">
+      <c r="AD374" t="inlineStr"/>
+      <c r="AE374" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45103,7 +46102,8 @@
       <c r="AA375" t="inlineStr"/>
       <c r="AB375" t="inlineStr"/>
       <c r="AC375" t="inlineStr"/>
-      <c r="AD375" t="inlineStr">
+      <c r="AD375" t="inlineStr"/>
+      <c r="AE375" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45211,7 +46211,8 @@
       <c r="AA376" t="inlineStr"/>
       <c r="AB376" t="inlineStr"/>
       <c r="AC376" t="inlineStr"/>
-      <c r="AD376" t="inlineStr">
+      <c r="AD376" t="inlineStr"/>
+      <c r="AE376" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45319,7 +46320,8 @@
       <c r="AA377" t="inlineStr"/>
       <c r="AB377" t="inlineStr"/>
       <c r="AC377" t="inlineStr"/>
-      <c r="AD377" t="inlineStr">
+      <c r="AD377" t="inlineStr"/>
+      <c r="AE377" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45431,7 +46433,8 @@
       <c r="AA378" t="inlineStr"/>
       <c r="AB378" t="inlineStr"/>
       <c r="AC378" t="inlineStr"/>
-      <c r="AD378" t="inlineStr">
+      <c r="AD378" t="inlineStr"/>
+      <c r="AE378" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45545,7 +46548,8 @@
       <c r="AA379" t="inlineStr"/>
       <c r="AB379" t="inlineStr"/>
       <c r="AC379" t="inlineStr"/>
-      <c r="AD379" t="inlineStr">
+      <c r="AD379" t="inlineStr"/>
+      <c r="AE379" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45667,7 +46671,8 @@
       <c r="AA380" t="inlineStr"/>
       <c r="AB380" t="inlineStr"/>
       <c r="AC380" t="inlineStr"/>
-      <c r="AD380" t="inlineStr">
+      <c r="AD380" t="inlineStr"/>
+      <c r="AE380" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45781,7 +46786,8 @@
       <c r="AA381" t="inlineStr"/>
       <c r="AB381" t="inlineStr"/>
       <c r="AC381" t="inlineStr"/>
-      <c r="AD381" t="inlineStr">
+      <c r="AD381" t="inlineStr"/>
+      <c r="AE381" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -45895,7 +46901,8 @@
       <c r="AA382" t="inlineStr"/>
       <c r="AB382" t="inlineStr"/>
       <c r="AC382" t="inlineStr"/>
-      <c r="AD382" t="inlineStr">
+      <c r="AD382" t="inlineStr"/>
+      <c r="AE382" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46009,7 +47016,8 @@
       <c r="AA383" t="inlineStr"/>
       <c r="AB383" t="inlineStr"/>
       <c r="AC383" t="inlineStr"/>
-      <c r="AD383" t="inlineStr">
+      <c r="AD383" t="inlineStr"/>
+      <c r="AE383" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46077,7 +47085,8 @@
       <c r="AA384" t="inlineStr"/>
       <c r="AB384" t="inlineStr"/>
       <c r="AC384" t="inlineStr"/>
-      <c r="AD384" t="inlineStr">
+      <c r="AD384" t="inlineStr"/>
+      <c r="AE384" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46182,7 +47191,8 @@
       <c r="AA385" t="inlineStr"/>
       <c r="AB385" t="inlineStr"/>
       <c r="AC385" t="inlineStr"/>
-      <c r="AD385" t="inlineStr">
+      <c r="AD385" t="inlineStr"/>
+      <c r="AE385" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46302,7 +47312,8 @@
       <c r="AA386" t="inlineStr"/>
       <c r="AB386" t="inlineStr"/>
       <c r="AC386" t="inlineStr"/>
-      <c r="AD386" t="inlineStr">
+      <c r="AD386" t="inlineStr"/>
+      <c r="AE386" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46407,7 +47418,8 @@
       <c r="AA387" t="inlineStr"/>
       <c r="AB387" t="inlineStr"/>
       <c r="AC387" t="inlineStr"/>
-      <c r="AD387" t="inlineStr">
+      <c r="AD387" t="inlineStr"/>
+      <c r="AE387" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46521,7 +47533,8 @@
       <c r="AA388" t="inlineStr"/>
       <c r="AB388" t="inlineStr"/>
       <c r="AC388" t="inlineStr"/>
-      <c r="AD388" t="inlineStr">
+      <c r="AD388" t="inlineStr"/>
+      <c r="AE388" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46635,7 +47648,8 @@
       <c r="AA389" t="inlineStr"/>
       <c r="AB389" t="inlineStr"/>
       <c r="AC389" t="inlineStr"/>
-      <c r="AD389" t="inlineStr">
+      <c r="AD389" t="inlineStr"/>
+      <c r="AE389" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>
@@ -46719,7 +47733,8 @@
       <c r="AA390" t="inlineStr"/>
       <c r="AB390" t="inlineStr"/>
       <c r="AC390" t="inlineStr"/>
-      <c r="AD390" t="inlineStr">
+      <c r="AD390" t="inlineStr"/>
+      <c r="AE390" t="inlineStr">
         <is>
           <t>awaiting_review</t>
         </is>

</xml_diff>